<commit_message>
Inventory domain backend and tests implemented
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/orders/Performance Food/Performance Food_Bakery_20260707.xlsx
+++ b/WorkBot/main/data/orders/Performance Food/Performance Food_Bakery_20260707.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,6 +521,489 @@
         <v>25.8</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FC576</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Oil - Olive Extra Virgin</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>85.03</v>
+      </c>
+      <c r="E8" t="n">
+        <v>510.18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T0948</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Almond Milk</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>35.74</v>
+      </c>
+      <c r="E9" t="n">
+        <v>35.74</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BEH52</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Joe Tea - Raspberry</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E10" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AKJ06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Joe Tea - Half &amp; Half</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E11" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AKJ08</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Joe Tea - Classic Lemonade</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BEJ84</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Joe Tea - Black Cherry</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="E13" t="n">
+        <v>21.95</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>H2822</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Cannoli Shells - Large</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>34.17</v>
+      </c>
+      <c r="E14" t="n">
+        <v>34.17</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>23978</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Monin - Vanilla</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>37.89</v>
+      </c>
+      <c r="E15" t="n">
+        <v>37.89</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GK608</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Corn - Frozen</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>24.41</v>
+      </c>
+      <c r="E16" t="n">
+        <v>24.41</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CF124</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Half &amp; Half</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>25.09</v>
+      </c>
+      <c r="E17" t="n">
+        <v>50.18</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CM230</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Oat Milk</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="E18" t="n">
+        <v>78.25</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>J2280</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Yogurt - Plain (BIB)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>29.05</v>
+      </c>
+      <c r="E19" t="n">
+        <v>58.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E3556</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Pastrami (Sliced)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>68.56999999999999</v>
+      </c>
+      <c r="E20" t="n">
+        <v>68.56999999999999</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>WF580</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Corned Beef (Sliced)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>71.20999999999999</v>
+      </c>
+      <c r="E21" t="n">
+        <v>71.20999999999999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>HH264</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Muenster (Sliced)</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>48.07</v>
+      </c>
+      <c r="E22" t="n">
+        <v>96.14</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AV906</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Swiss (Sliced)</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>57.13</v>
+      </c>
+      <c r="E23" t="n">
+        <v>171.39</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CF096</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Fresh Mozz (Sliced)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>50.19</v>
+      </c>
+      <c r="E24" t="n">
+        <v>100.38</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>VR126</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cheddar - Extra Sharp White</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="E25" t="n">
+        <v>144.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>L9698</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Herb - Rosemary (Fresh)</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="E26" t="n">
+        <v>40.23</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>K1570</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Buttermilk</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="E27" t="n">
+        <v>18.38</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>G5010</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Carrots - Jumbo Fresh</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>42.51</v>
+      </c>
+      <c r="E28" t="n">
+        <v>42.51</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>FB270</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roma - Tiramisu Plastic Cup</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>34.79</v>
+      </c>
+      <c r="E29" t="n">
+        <v>34.79</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>FB268</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Mousse Cup - Chocolate</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>32.26</v>
+      </c>
+      <c r="E30" t="n">
+        <v>32.26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>